<commit_message>
📝 docs(WBS): 시험 단계 85%→95% — 5.4 보안 완료(100)·5.5 성능 CRITICAL 종결(90)
- 5.4: KISA IE·IL·MC 추가확인 3항목 완결 → 21항목 전체 양호, 상태 완료
- 5.5: 잔여 CRITICAL 3건 재검증 종결(PRD_18 v1.1), 잔여=라운드6+ HIGH/MED
- 5 종합 95% — 잔여는 5.3 PyVoice S0 실기기 검증(마스터 실기기 필요)뿐

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wbs_new.xlsx
+++ b/docs/wbs_new.xlsx
@@ -2741,7 +2741,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr"/>
       <c r="H47" s="5" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
@@ -2925,20 +2925,20 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>진행중</t>
+        <v>100</v>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>🔍 추가확인 3항목 잔여</t>
+          <t>2026-07-08 IE·IL·MC 3항목 완결 — 21항목 전체 양호 (IE del_yn 차단 복원·IL 39지점 정제·MC Magic Byte 5경로)</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr"/>
       <c r="H52" s="7" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>잔여 CRITICAL 3건</t>
+          <t>CRITICAL 0건 (3건 재검증 종결 2026-07-08, PRD_18 v1.1) — 잔여 라운드6+ HIGH/MED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📝 docs(분석·WBS): PRD_21 v1.2 구현 실사 현행화 + WBS 구현 96% 갱신 + 지표 모수 del_yn 보정
- PRD_21: §7-0 실사 표 신설(4탭 설계기준 85%·6도메인 68%), §6 온더플라이 설계변경
  명문화(코호트·RFM 사전집계 미채택), §12-3④ 퍼포먼스 탭 '선결 대기'→'실가동' 격상
  (stat_pageview 수집층), §12-5 stats 병존 실태 기록
- WBS: 4.19·4.21→100%(완료일 07-08), 4.25→85%(기획→진행중), 4.26→90%,
  구현 대분류 92→96%, 요약 전체 진척률 약 91%
- 지표 정확성: analytics usage(가입자·코호트 모수)·performance(전환율 분모)에
  sys_user del_yn='N' 필터 추가 — 'del_yn 없음' 낡은 전제(sql/127 이전) 제거

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wbs_new.xlsx
+++ b/docs/wbs_new.xlsx
@@ -1455,7 +1455,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr"/>
       <c r="H20" s="5" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
@@ -2365,11 +2365,11 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>잔여: 보상 A2U(이벤트·캠페인) 미전환</t>
+          <t>✅잔여였던 보상 A2U(이벤트·캠페인) 완결 — 관리자 승인 게이트·sql/171 (07-08, 운영DB 적용 대기)</t>
         </is>
       </c>
     </row>
@@ -2465,11 +2465,11 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>잔여: 통합알림(TXN_ST/FBCK) 트리거</t>
+          <t>✅잔여였던 통합알림(TXN_ST/FBCK) 완결 — trade-noti·기존 1분 cron 재사용 (07-08)</t>
         </is>
       </c>
     </row>
@@ -2661,16 +2661,16 @@
       </c>
       <c r="G45" s="7" t="inlineStr"/>
       <c r="H45" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="I45" s="10" t="inlineStr">
-        <is>
-          <t>기획</t>
+        <v>85</v>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>진행중</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>구현 대기·sql/122~125 제안</t>
+          <t>4탭 구현·운영 중(설계기준 85% — 07-08 실사·PRD_21 v1.2) — 잔여: 지리 지도·채널 퍼널·내보내기</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr"/>
       <c r="H46" s="7" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="I46" s="9" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>미결정: 저장·보존·갱신주기</t>
+          <t>보존 7일 cron(sql/170)·미결정 3건 확정(07-08, PRD_22 v1.1) — 잔여: Vercel Analytics·RPC 2종</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>약 90% — 구현 Phase 0~28 중 24개 완료, 등재·모니터링·분석 잔여</t>
+          <t>약 91% — 구현 96%(26개 작업 중 22개 완료), 최우선 잔여=메인넷 등재(6.4)·운영 안정화</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-08 (자동 생성 — PRD·ROADMAP 라이트버전 기반)</t>
+          <t>2026-07-08 (자동 생성 — PRD·ROADMAP 라이트버전 기반 · 07-08 구현 실사 현행화)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📝 docs(현행화): 2026-07-09 4트랙 실적 종합 — PRD v13.1·ROADMAP v13.1·WBS 65행 갱신
- ROADMAP: 법무·횡단9차 행 신설 + Phase 22(P1 적용)·24(등재 준비 가속) 갱신 + 변경 이력 v13.1
- PRD: #43 i18n 에러코드 완결·#44 법무 4종 v1.1 신설, #33 분석 🚧 전환
- WBS: 4.27(횡단9 ✅)·4.28(팩토리 ⏸️보류) 신설, 법무 95%·성능시험 70%·메인넷 등재 60%·전체 ~92%

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wbs_new.xlsx
+++ b/docs/wbs_new.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="355">
   <si>
     <t>WBS ID</t>
   </si>
@@ -146,7 +146,7 @@
     <t>2026-06-12</t>
   </si>
   <si>
-    <t>v1.1 초안 완료(kor/eng)·공지 후 7/15 시행 예정·T05 외부 회신 대기</t>
+    <t>4종 v1.1(방침·환불·약관·커뮤니티) 공지 3건 게시 완료·7/16 promote로 시행·잔여 T05 외부·G-8/9 경미</t>
   </si>
   <si>
     <t>2</t>
@@ -335,7 +335,7 @@
     <t>구현</t>
   </si>
   <si>
-    <t>Phase 0~28</t>
+    <t>Phase 0~29 + 횡단 9차</t>
   </si>
   <si>
     <t>4.1</t>
@@ -719,7 +719,7 @@
     <t>PRD_21_DATA_ANAL</t>
   </si>
   <si>
-    <t>구현 대기·sql/122~125 제안</t>
+    <t>P1 적용(매출 탭 KPI 델타·오늘 실시간 매출, 07-08)·잔여 탭 3종</t>
   </si>
   <si>
     <t>4.26</t>
@@ -737,6 +737,42 @@
     <t>미결정: 저장·보존·갱신주기</t>
   </si>
   <si>
+    <t>4.27</t>
+  </si>
+  <si>
+    <t>i18n 완결</t>
+  </si>
+  <si>
+    <t>횡단 9차 — 하드코딩 한국어 전수 제거 + API 에러코드 i18n (107 route 587지점·admin 82파일·1,633키×66언어)</t>
+  </si>
+  <si>
+    <t>i18n 감사 정본</t>
+  </si>
+  <si>
+    <t>2026-07-09</t>
+  </si>
+  <si>
+    <t>감사 잔여 0건·ESLint 91→0</t>
+  </si>
+  <si>
+    <t>4.28</t>
+  </si>
+  <si>
+    <t>팩토리</t>
+  </si>
+  <si>
+    <t>Phase 29 Pi 앱 팩토리 — .pi 도메인 멀티테넌트 (설계·도메인 19개 매핑·yea.pi 컨셉·sql/173 초안)</t>
+  </si>
+  <si>
+    <t>PRD_27_PI_FACTORY v1.3</t>
+  </si>
+  <si>
+    <t>보류</t>
+  </si>
+  <si>
+    <t>⏸️무기한 홀딩(마스터) — 가능성 타진 완료·구현 착수 금지·모선 집중</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
@@ -812,7 +848,7 @@
     <t>PRD_18_PERFORM·troubleshoot/PERF_*</t>
   </si>
   <si>
-    <t>잔여 CRITICAL 3건</t>
+    <t>SHOP window.Pi 가드 검증 종결(07-09)·잔여 CRITICAL 2건(CAFE WebSocket·MAP 클러스터링)</t>
   </si>
   <si>
     <t>5.6</t>
@@ -890,7 +926,7 @@
     <t>MAINNET_READINESS_CHECKLIST.md</t>
   </si>
   <si>
-    <t>⭐ 최우선 잔여 과제</t>
+    <t>⭐최우선 — 절제 오버레이 운영 검증(C-1-F-①)·listing prep/live(sql/169·172)·방침 A-7 입증 완결(07-09). 잔여=포털 수작업·신청</t>
   </si>
   <si>
     <t>7</t>
@@ -1010,7 +1046,7 @@
     <t>전체 진척률</t>
   </si>
   <si>
-    <t>약 90% — 구현 Phase 0~28 중 24개 완료, 등재·모니터링·분석 잔여</t>
+    <t>약 92% — 구현 26개 완료(횡단 9차 포함)·법무 4종 v1.1 공지 완료(7/16 시행)·팩토리 홀딩. 잔여: 메인넷 등재(60%)·모니터링·분석·성능 CRITICAL 2건</t>
   </si>
   <si>
     <t>핵심 가치</t>
@@ -1040,7 +1076,7 @@
     <t>작성일</t>
   </si>
   <si>
-    <t>2026-07-08 (자동 생성 — PRD·ROADMAP 라이트버전 기반)</t>
+    <t>2026-07-09 갱신 (자동 생성 — PRD v13.1·ROADMAP v13.1 기반)</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1099,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1097,6 +1133,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFEFEFEF"/>
       </patternFill>
     </fill>
@@ -1120,7 +1161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1149,6 +1190,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1493,7 +1537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1721,7 +1765,7 @@
         <v>12</v>
       </c>
       <c r="H7" s="7">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>14</v>
@@ -2137,7 +2181,7 @@
         <v>12</v>
       </c>
       <c r="H20" s="5">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>14</v>
@@ -2937,10 +2981,10 @@
         <v>12</v>
       </c>
       <c r="H45" s="7">
-        <v>20</v>
-      </c>
-      <c r="I45" s="10" t="s">
-        <v>185</v>
+        <v>40</v>
+      </c>
+      <c r="I45" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="J45" s="6" t="s">
         <v>235</v>
@@ -2978,213 +3022,213 @@
         <v>240</v>
       </c>
     </row>
-    <row r="47" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="4" t="s">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="C47" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H47" s="5">
-        <v>85</v>
-      </c>
-      <c r="I47" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>12</v>
+      <c r="D47" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="H47" s="7">
+        <v>100</v>
+      </c>
+      <c r="I47" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>242</v>
+        <v>106</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D48" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="F48" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="E48" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="F48" s="7" t="s">
+      <c r="G48" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="H48" s="7">
+        <v>15</v>
+      </c>
+      <c r="I48" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F49" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G48" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H48" s="7">
-        <v>100</v>
-      </c>
-      <c r="I48" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J48" s="6" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="F49" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H49" s="7">
-        <v>100</v>
-      </c>
-      <c r="I49" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J49" s="6" t="s">
+      <c r="G49" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" s="5">
+        <v>85</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J49" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="H50" s="7">
-        <v>95</v>
-      </c>
-      <c r="I50" s="9" t="s">
-        <v>14</v>
+        <v>100</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>63</v>
+        <v>158</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="H51" s="7">
-        <v>90</v>
-      </c>
-      <c r="I51" s="9" t="s">
-        <v>14</v>
+        <v>100</v>
+      </c>
+      <c r="I51" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>261</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="H52" s="7">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="I52" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>63</v>
@@ -3193,132 +3237,132 @@
         <v>63</v>
       </c>
       <c r="H53" s="7">
-        <v>100</v>
-      </c>
-      <c r="I53" s="8" t="s">
-        <v>21</v>
+        <v>90</v>
+      </c>
+      <c r="I53" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="B54" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="C54" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H54" s="5">
-        <v>80</v>
-      </c>
-      <c r="I54" s="5" t="s">
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H54" s="7">
+        <v>70</v>
+      </c>
+      <c r="I54" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J54" s="4" t="s">
-        <v>12</v>
+      <c r="J54" s="6" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>273</v>
+        <v>254</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="F55" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H55" s="7">
+        <v>100</v>
+      </c>
+      <c r="I55" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J55" s="6" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F56" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G55" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="H55" s="7">
-        <v>100</v>
-      </c>
-      <c r="I55" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J55" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="H56" s="7">
-        <v>100</v>
-      </c>
-      <c r="I56" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J56" s="6" t="s">
-        <v>282</v>
+      <c r="G56" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H56" s="5">
+        <v>85</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>230</v>
+        <v>202</v>
       </c>
       <c r="H57" s="7">
         <v>100</v>
@@ -3327,94 +3371,94 @@
         <v>21</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>287</v>
+        <v>12</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>213</v>
+        <v>78</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>12</v>
+        <v>202</v>
       </c>
       <c r="H58" s="7">
-        <v>40</v>
-      </c>
-      <c r="I58" s="9" t="s">
-        <v>14</v>
+        <v>100</v>
+      </c>
+      <c r="I58" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="B59" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="C59" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F59" s="5" t="s">
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="F59" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="G59" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H59" s="5">
-        <v>60</v>
-      </c>
-      <c r="I59" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="J59" s="4" t="s">
-        <v>12</v>
+      <c r="G59" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="H59" s="7">
+        <v>100</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J59" s="6" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>47</v>
+        <v>213</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>299</v>
+        <v>12</v>
       </c>
       <c r="H60" s="7">
         <v>60</v>
@@ -3423,134 +3467,198 @@
         <v>14</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="E61" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="F61" s="7" t="s">
+    </row>
+    <row r="61" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F61" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G61" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H61" s="7">
-        <v>70</v>
-      </c>
-      <c r="I61" s="9" t="s">
+      <c r="G61" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H61" s="5">
+        <v>60</v>
+      </c>
+      <c r="I61" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J61" s="6" t="s">
-        <v>305</v>
+      <c r="J61" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>294</v>
-      </c>
       <c r="C62" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>310</v>
+        <v>47</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>12</v>
+        <v>311</v>
       </c>
       <c r="H62" s="7">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I62" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>12</v>
+        <v>312</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>147</v>
+        <v>47</v>
       </c>
       <c r="G63" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H63" s="7">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="I63" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>12</v>
+        <v>322</v>
       </c>
       <c r="G64" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H64" s="7">
+        <v>50</v>
+      </c>
+      <c r="I64" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J64" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="F65" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="G65" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H65" s="7">
+        <v>30</v>
+      </c>
+      <c r="I65" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J65" s="6" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H66" s="7">
         <v>0</v>
       </c>
-      <c r="I64" s="11" t="s">
-        <v>320</v>
-      </c>
-      <c r="J64" s="6" t="s">
+      <c r="I66" s="12" t="s">
+        <v>332</v>
+      </c>
+      <c r="J66" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3571,91 +3679,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
-        <v>321</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>322</v>
+      <c r="A1" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📝 docs(현행화): 2026-07-10 종합 — PRD·ROADMAP v13.3 (하네스의 날, 14커밋·4트랙)
- 하네스 2종 실전(등록팀·DA팀 5인)·등재 제출 직전 단계(잔여=포털 5건)·전수감사 PASS·접두사 22종·번역 오염 근본수정·보안 재발 방지 종합
- ROADMAP 하네스 행 신설·Phase 24 갱신 / PRD #45·#46 신설 / WBS 66행(4.29 하네스·6.4 등재 70%)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wbs_new.xlsx
+++ b/docs/wbs_new.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="361">
   <si>
     <t>WBS ID</t>
   </si>
@@ -194,123 +194,126 @@
     <t>데이터 표준</t>
   </si>
   <si>
-    <t>DA 표준 규칙·표준사전·품질점검기준 수립</t>
-  </si>
-  <si>
-    <t>docs/da/데이터표준규칙.md·품질점검기준서.md</t>
+    <t>DA 표준 규칙·표준사전·품질점검기준 수립·운영</t>
+  </si>
+  <si>
+    <t>docs/da/데이터표준규칙.md·reports/</t>
   </si>
   <si>
     <t>2026-06-06</t>
   </si>
   <si>
+    <t>2026-07-10</t>
+  </si>
+  <si>
+    <t>전수감사 2차(sql/102~175 PASS, da-team 하네스)·접두사 22종 현행화</t>
+  </si>
+  <si>
+    <t>2.4</t>
+  </si>
+  <si>
+    <t>제약사항 분석</t>
+  </si>
+  <si>
+    <t>Pi Browser WebView 제약·Vercel·NextAuth beta 제약 정의</t>
+  </si>
+  <si>
+    <t>ROADMAP §운영 인프라 제약·CLAUDE.md</t>
+  </si>
+  <si>
+    <t>2026-06-18</t>
+  </si>
+  <si>
+    <t>Set-Cookie 미저장→이중 경로 확정</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>설계</t>
+  </si>
+  <si>
+    <t>2026-06-25</t>
+  </si>
+  <si>
+    <t>3.1</t>
+  </si>
+  <si>
+    <t>아키텍처 설계</t>
+  </si>
+  <si>
+    <t>Next.js 16 + Supabase + Pi SDK 구조·3-tier DB 라우터</t>
+  </si>
+  <si>
+    <t>docs/PRD.md §1·INFRA_DB_TIERS.md·src/lib/db-env.ts</t>
+  </si>
+  <si>
+    <t>2026-06-28</t>
+  </si>
+  <si>
+    <t>2단계 배포(staging→운영) 분리</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>인증 설계</t>
+  </si>
+  <si>
+    <t>쿠키+X-Pi-Token 이중 경로·클라이언트 게이트·Pi Sign-In OAuth</t>
+  </si>
+  <si>
+    <t>CLAUDE.md 인증+세션 구조</t>
+  </si>
+  <si>
+    <t>UA 사전차단 금지 철칙 포함</t>
+  </si>
+  <si>
+    <t>3.3</t>
+  </si>
+  <si>
+    <t>DB 설계</t>
+  </si>
+  <si>
+    <t>96테이블 스키마·DA 표준(시스템컬럼4·논리삭제)·FK 정책</t>
+  </si>
+  <si>
+    <t>sql/*.sql·PRD.md §6</t>
+  </si>
+  <si>
+    <t>sql/001~168</t>
+  </si>
+  <si>
+    <t>3.4</t>
+  </si>
+  <si>
+    <t>UI/UX 설계</t>
+  </si>
+  <si>
+    <t>Tailwind v4 + base-nova·다크모드·반응형 목록 표준</t>
+  </si>
+  <si>
+    <t>CLAUDE.md 프론트엔드 표준</t>
+  </si>
+  <si>
+    <t>페이지네이션·lazy 로딩 3원칙</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>보안 설계</t>
+  </si>
+  <si>
+    <t>KISA 21항목 분석·DDoS 5계층 방어 아키텍처</t>
+  </si>
+  <si>
+    <t>docs/PRD_2_SECURITY.md·SECURITY_DDOS_POLICY.md</t>
+  </si>
+  <si>
     <t>2026-06-23</t>
   </si>
   <si>
-    <t>횡단7차 전수감사 준수율 100%</t>
-  </si>
-  <si>
-    <t>2.4</t>
-  </si>
-  <si>
-    <t>제약사항 분석</t>
-  </si>
-  <si>
-    <t>Pi Browser WebView 제약·Vercel·NextAuth beta 제약 정의</t>
-  </si>
-  <si>
-    <t>ROADMAP §운영 인프라 제약·CLAUDE.md</t>
-  </si>
-  <si>
-    <t>2026-06-18</t>
-  </si>
-  <si>
-    <t>Set-Cookie 미저장→이중 경로 확정</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>설계</t>
-  </si>
-  <si>
-    <t>2026-06-25</t>
-  </si>
-  <si>
-    <t>3.1</t>
-  </si>
-  <si>
-    <t>아키텍처 설계</t>
-  </si>
-  <si>
-    <t>Next.js 16 + Supabase + Pi SDK 구조·3-tier DB 라우터</t>
-  </si>
-  <si>
-    <t>docs/PRD.md §1·INFRA_DB_TIERS.md·src/lib/db-env.ts</t>
-  </si>
-  <si>
-    <t>2026-06-28</t>
-  </si>
-  <si>
-    <t>2단계 배포(staging→운영) 분리</t>
-  </si>
-  <si>
-    <t>3.2</t>
-  </si>
-  <si>
-    <t>인증 설계</t>
-  </si>
-  <si>
-    <t>쿠키+X-Pi-Token 이중 경로·클라이언트 게이트·Pi Sign-In OAuth</t>
-  </si>
-  <si>
-    <t>CLAUDE.md 인증+세션 구조</t>
-  </si>
-  <si>
-    <t>UA 사전차단 금지 철칙 포함</t>
-  </si>
-  <si>
-    <t>3.3</t>
-  </si>
-  <si>
-    <t>DB 설계</t>
-  </si>
-  <si>
-    <t>96테이블 스키마·DA 표준(시스템컬럼4·논리삭제)·FK 정책</t>
-  </si>
-  <si>
-    <t>sql/*.sql·PRD.md §6</t>
-  </si>
-  <si>
-    <t>sql/001~168</t>
-  </si>
-  <si>
-    <t>3.4</t>
-  </si>
-  <si>
-    <t>UI/UX 설계</t>
-  </si>
-  <si>
-    <t>Tailwind v4 + base-nova·다크모드·반응형 목록 표준</t>
-  </si>
-  <si>
-    <t>CLAUDE.md 프론트엔드 표준</t>
-  </si>
-  <si>
-    <t>페이지네이션·lazy 로딩 3원칙</t>
-  </si>
-  <si>
-    <t>3.5</t>
-  </si>
-  <si>
-    <t>보안 설계</t>
-  </si>
-  <si>
-    <t>KISA 21항목 분석·DDoS 5계층 방어 아키텍처</t>
-  </si>
-  <si>
-    <t>docs/PRD_2_SECURITY.md·SECURITY_DDOS_POLICY.md</t>
-  </si>
-  <si>
     <t>✅18 양호·🔍3 추가확인</t>
   </si>
   <si>
@@ -722,9 +725,6 @@
     <t>PRD_21_DATA_ANAL</t>
   </si>
   <si>
-    <t>2026-07-10</t>
-  </si>
-  <si>
     <t>4탭 전부 운영 중(실사 v1.2)+CSV 내보내기(07-10). 잔여=퍼널·지리(선결 대기)</t>
   </si>
   <si>
@@ -758,6 +758,21 @@
     <t>감사 잔여 0건·ESLint 91→0</t>
   </si>
   <si>
+    <t>4.29</t>
+  </si>
+  <si>
+    <t>하네스</t>
+  </si>
+  <si>
+    <t>멀티에이전트 팀 2종 — 메인넷 등록팀(4역할·재실행 가능)·DA팀 5인(da-team 스킬·전수감사·설계 실전)</t>
+  </si>
+  <si>
+    <t>.claude/workflows·CLAUDE.md 하네스 절</t>
+  </si>
+  <si>
+    <t>등재 런북·전수감사 PASS·sys_cfg_chg_hist 설계 산출</t>
+  </si>
+  <si>
     <t>4.28</t>
   </si>
   <si>
@@ -929,7 +944,7 @@
     <t>MAINNET_READINESS_CHECKLIST.md</t>
   </si>
   <si>
-    <t>⭐최우선 — 절제 오버레이 운영 검증(C-1-F-①)·listing prep/live(sql/169·172)·방침 A-7 입증 완결(07-09). 잔여=포털 수작업·신청</t>
+    <t>⭐제출 직전 — 실행 런북 확정(7단+P0 12단계, 07-10 등록팀 하네스)·부록 현행화·레드라인 전부 OK 실측. 잔여=마스터 포털 5건뿐</t>
   </si>
   <si>
     <t>7</t>
@@ -1540,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2114,10 +2129,10 @@
         <v>98</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="H18" s="7">
         <v>100</v>
@@ -2126,24 +2141,24 @@
         <v>21</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>72</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>69</v>
@@ -2158,15 +2173,15 @@
         <v>21</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>12</v>
@@ -2190,24 +2205,24 @@
         <v>14</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>13</v>
@@ -2227,19 +2242,19 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>13</v>
@@ -2254,24 +2269,24 @@
         <v>21</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>13</v>
@@ -2291,19 +2306,19 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>13</v>
@@ -2323,19 +2338,19 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>13</v>
@@ -2355,19 +2370,19 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>59</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>62</v>
@@ -2387,25 +2402,25 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H27" s="7">
         <v>100</v>
@@ -2414,30 +2429,30 @@
         <v>21</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H28" s="7">
         <v>100</v>
@@ -2451,25 +2466,25 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H29" s="7">
         <v>100</v>
@@ -2483,25 +2498,25 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F30" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>147</v>
-      </c>
       <c r="G30" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H30" s="7">
         <v>100</v>
@@ -2510,27 +2525,27 @@
         <v>21</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G31" s="7" t="s">
         <v>43</v>
@@ -2542,30 +2557,30 @@
         <v>21</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H32" s="7">
         <v>100</v>
@@ -2574,24 +2589,24 @@
         <v>21</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>43</v>
@@ -2606,24 +2621,24 @@
         <v>21</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>43</v>
@@ -2638,30 +2653,30 @@
         <v>21</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H35" s="7">
         <v>100</v>
@@ -2670,27 +2685,27 @@
         <v>21</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>12</v>
@@ -2699,27 +2714,27 @@
         <v>30</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>69</v>
@@ -2739,25 +2754,25 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H38" s="7">
         <v>90</v>
@@ -2766,27 +2781,27 @@
         <v>14</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>47</v>
@@ -2798,24 +2813,24 @@
         <v>21</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>47</v>
@@ -2830,30 +2845,30 @@
         <v>21</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H41" s="7">
         <v>100</v>
@@ -2862,27 +2877,27 @@
         <v>21</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G42" s="7" t="s">
         <v>32</v>
@@ -2894,24 +2909,24 @@
         <v>21</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>32</v>
@@ -2926,30 +2941,30 @@
         <v>21</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>43</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H44" s="7">
         <v>100</v>
@@ -2963,25 +2978,25 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>73</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>236</v>
+        <v>63</v>
       </c>
       <c r="H45" s="7">
         <v>95</v>
@@ -2998,7 +3013,7 @@
         <v>238</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>239</v>
@@ -3013,7 +3028,7 @@
         <v>73</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H46" s="7">
         <v>85</v>
@@ -3030,7 +3045,7 @@
         <v>243</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>244</v>
@@ -3045,7 +3060,7 @@
         <v>32</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H47" s="7">
         <v>100</v>
@@ -3062,7 +3077,7 @@
         <v>248</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>249</v>
@@ -3074,83 +3089,83 @@
         <v>251</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>214</v>
+        <v>63</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>214</v>
+        <v>63</v>
       </c>
       <c r="H48" s="7">
+        <v>100</v>
+      </c>
+      <c r="I48" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="H49" s="7">
         <v>15</v>
       </c>
-      <c r="I48" s="11" t="s">
-        <v>252</v>
-      </c>
-      <c r="J48" s="6" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F49" s="5" t="s">
+      <c r="I49" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G49" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H49" s="5">
+      <c r="G50" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H50" s="5">
         <v>85</v>
       </c>
-      <c r="I49" s="5" t="s">
+      <c r="I50" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J49" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H50" s="7">
-        <v>100</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>260</v>
+      <c r="J50" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
@@ -3158,7 +3173,7 @@
         <v>261</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>262</v>
@@ -3170,10 +3185,10 @@
         <v>264</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>158</v>
+        <v>13</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="H51" s="7">
         <v>100</v>
@@ -3182,39 +3197,39 @@
         <v>21</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>12</v>
+        <v>265</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>13</v>
+        <v>159</v>
       </c>
       <c r="G52" s="7" t="s">
         <v>32</v>
       </c>
       <c r="H52" s="7">
-        <v>95</v>
-      </c>
-      <c r="I52" s="9" t="s">
-        <v>14</v>
+        <v>100</v>
+      </c>
+      <c r="I52" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>269</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
@@ -3222,7 +3237,7 @@
         <v>270</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>271</v>
@@ -3234,13 +3249,13 @@
         <v>273</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="H53" s="7">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I53" s="9" t="s">
         <v>14</v>
@@ -3254,7 +3269,7 @@
         <v>275</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>276</v>
@@ -3266,10 +3281,10 @@
         <v>278</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>214</v>
+        <v>99</v>
       </c>
       <c r="H54" s="7">
         <v>90</v>
@@ -3286,7 +3301,7 @@
         <v>280</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>281</v>
@@ -3298,106 +3313,106 @@
         <v>283</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>63</v>
+        <v>215</v>
       </c>
       <c r="H55" s="7">
-        <v>100</v>
-      </c>
-      <c r="I55" s="8" t="s">
-        <v>21</v>
+        <v>90</v>
+      </c>
+      <c r="I55" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="J55" s="6" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="56" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="C56" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F56" s="5" t="s">
+      <c r="D56" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="H56" s="7">
+        <v>100</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J56" s="6" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F57" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G56" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H56" s="5">
+      <c r="G57" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H57" s="5">
         <v>85</v>
       </c>
-      <c r="I56" s="5" t="s">
+      <c r="I57" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J56" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>288</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G57" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="H57" s="7">
-        <v>100</v>
-      </c>
-      <c r="I57" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J57" s="6" t="s">
+      <c r="J57" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B58" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="B58" s="6" t="s">
-        <v>286</v>
-      </c>
       <c r="C58" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H58" s="7">
         <v>100</v>
@@ -3406,7 +3421,7 @@
         <v>21</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>295</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -3414,7 +3429,7 @@
         <v>296</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>297</v>
@@ -3426,10 +3441,10 @@
         <v>299</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>231</v>
+        <v>203</v>
       </c>
       <c r="H59" s="7">
         <v>100</v>
@@ -3446,7 +3461,7 @@
         <v>301</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>302</v>
@@ -3458,109 +3473,109 @@
         <v>304</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>213</v>
+        <v>47</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>12</v>
+        <v>232</v>
       </c>
       <c r="H60" s="7">
-        <v>60</v>
-      </c>
-      <c r="I60" s="9" t="s">
-        <v>14</v>
+        <v>100</v>
+      </c>
+      <c r="I60" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="J60" s="6" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="61" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C61" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="C61" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E61" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F61" s="5" t="s">
+      <c r="D61" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H61" s="7">
+        <v>70</v>
+      </c>
+      <c r="I61" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J61" s="6" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F62" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G61" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H61" s="5">
+      <c r="G62" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H62" s="5">
         <v>60</v>
       </c>
-      <c r="I61" s="5" t="s">
+      <c r="I62" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J61" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="6" t="s">
-        <v>308</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="D62" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="F62" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G62" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="H62" s="7">
-        <v>60</v>
-      </c>
-      <c r="I62" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J62" s="6" t="s">
-        <v>313</v>
+      <c r="J62" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C63" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="C63" s="6" t="s">
+      <c r="D63" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="D63" s="6" t="s">
+      <c r="E63" s="6" t="s">
         <v>316</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>317</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>47</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>12</v>
+        <v>317</v>
       </c>
       <c r="H63" s="7">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I63" s="9" t="s">
         <v>14</v>
@@ -3574,7 +3589,7 @@
         <v>319</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>320</v>
@@ -3586,19 +3601,19 @@
         <v>322</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>323</v>
+        <v>47</v>
       </c>
       <c r="G64" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H64" s="7">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="I64" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>12</v>
+        <v>323</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
@@ -3606,7 +3621,7 @@
         <v>324</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>325</v>
@@ -3618,19 +3633,19 @@
         <v>327</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>147</v>
+        <v>328</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H65" s="7">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I65" s="9" t="s">
         <v>14</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>328</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
@@ -3638,7 +3653,7 @@
         <v>329</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>330</v>
@@ -3650,18 +3665,50 @@
         <v>332</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>12</v>
+        <v>148</v>
       </c>
       <c r="G66" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H66" s="7">
+        <v>30</v>
+      </c>
+      <c r="I66" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="F67" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G67" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H67" s="7">
         <v>0</v>
       </c>
-      <c r="I66" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="J66" s="6" t="s">
+      <c r="I67" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="J67" s="6" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3683,90 +3730,90 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>